<commit_message>
ML DAY 1 PRACTICAL
</commit_message>
<xml_diff>
--- a/Basic of excel.xlsx
+++ b/Basic of excel.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="96" yWindow="144" windowWidth="23892" windowHeight="9768" activeTab="4"/>
+    <workbookView xWindow="96" yWindow="144" windowWidth="23256" windowHeight="9768" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="students" sheetId="4" r:id="rId1"/>
@@ -18,10 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>no</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Name</t>
   </si>
@@ -45,13 +42,55 @@
   </si>
   <si>
     <t>MATH.</t>
+  </si>
+  <si>
+    <t>AMIT</t>
+  </si>
+  <si>
+    <t>DILIP</t>
+  </si>
+  <si>
+    <t>RAMESH</t>
+  </si>
+  <si>
+    <t>HARKISHAN</t>
+  </si>
+  <si>
+    <t>RAJU</t>
+  </si>
+  <si>
+    <t>MAHENDRA</t>
+  </si>
+  <si>
+    <t>GIRISH</t>
+  </si>
+  <si>
+    <t>ASHOK</t>
+  </si>
+  <si>
+    <t>KALPESH</t>
+  </si>
+  <si>
+    <t>percentage</t>
+  </si>
+  <si>
+    <t>STUDENT MARSHEET OF DIVISION A 2026-27</t>
+  </si>
+  <si>
+    <t>PARAM AMITBHAI PATEL</t>
+  </si>
+  <si>
+    <t>DOB</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="[$-14009]dddd\,\ d\ mmmm\,\ yyyy;@"/>
+  </numFmts>
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -59,16 +98,58 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Berlin Sans FB"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Open Sans"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Inter"/>
+    </font>
+    <font>
+      <b/>
+      <u val="double"/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Open Sans"/>
+    </font>
+    <font>
+      <b/>
+      <u val="double"/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Lora"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Bookman Old Style"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -76,12 +157,61 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -427,44 +557,467 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A2:I2"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" customWidth="1"/>
-    <col min="3" max="9" width="5.33203125" customWidth="1"/>
+    <col min="1" max="1" width="4.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9">
-      <c r="A2" t="s">
+    <row r="1" spans="1:11" ht="24.6" customHeight="1">
+      <c r="A1" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+    </row>
+    <row r="2" spans="1:11" ht="23.4" customHeight="1">
+      <c r="A2" s="7"/>
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
+      <c r="H2" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="22.2">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="C3" s="13">
+        <v>27590</v>
+      </c>
+      <c r="D3" s="5">
+        <v>72</v>
+      </c>
+      <c r="E3" s="5">
+        <v>58</v>
+      </c>
+      <c r="F3" s="5">
+        <v>88</v>
+      </c>
+      <c r="G3" s="5">
+        <v>90</v>
+      </c>
+      <c r="H3" s="5">
+        <v>37</v>
+      </c>
+      <c r="I3" s="5">
+        <v>83</v>
+      </c>
+      <c r="J3" s="5">
+        <f>SUM(D3:I3)</f>
+        <v>428</v>
+      </c>
+      <c r="K3" s="6">
+        <f>J3/6</f>
+        <v>71.333333333333329</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="22.2">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="13">
+        <v>31284</v>
+      </c>
+      <c r="D4" s="5">
+        <v>45</v>
+      </c>
+      <c r="E4" s="5">
+        <v>67</v>
+      </c>
+      <c r="F4" s="5">
+        <v>64</v>
+      </c>
+      <c r="G4" s="5">
+        <v>50</v>
+      </c>
+      <c r="H4" s="5">
+        <v>65</v>
+      </c>
+      <c r="I4" s="5">
+        <v>54</v>
+      </c>
+      <c r="J4" s="5">
+        <f>SUM(D4:I4)</f>
+        <v>345</v>
+      </c>
+      <c r="K4" s="6">
+        <f>J4/6</f>
+        <v>57.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="22.2">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="13">
+        <v>34769</v>
+      </c>
+      <c r="D5" s="5">
+        <v>74</v>
+      </c>
+      <c r="E5" s="5">
+        <v>74</v>
+      </c>
+      <c r="F5" s="5">
+        <v>78</v>
+      </c>
+      <c r="G5" s="5">
+        <v>97</v>
+      </c>
+      <c r="H5" s="5">
+        <v>66</v>
+      </c>
+      <c r="I5" s="5">
+        <v>99</v>
+      </c>
+      <c r="J5" s="5">
+        <f>SUM(D5:I5)</f>
+        <v>488</v>
+      </c>
+      <c r="K5" s="6">
+        <f>J5/6</f>
+        <v>81.333333333333329</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="22.2">
+      <c r="A6" s="4">
+        <v>4</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="13">
+        <v>27587</v>
+      </c>
+      <c r="D6" s="5">
+        <v>45</v>
+      </c>
+      <c r="E6" s="5">
+        <v>68</v>
+      </c>
+      <c r="F6" s="5">
+        <v>83</v>
+      </c>
+      <c r="G6" s="5">
+        <v>48</v>
+      </c>
+      <c r="H6" s="5">
+        <v>66</v>
+      </c>
+      <c r="I6" s="5">
+        <v>44</v>
+      </c>
+      <c r="J6" s="5">
+        <f>SUM(D6:I6)</f>
+        <v>354</v>
+      </c>
+      <c r="K6" s="6">
+        <f>AVERAGE(D6:I6)</f>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="22.2">
+      <c r="A7" s="4">
+        <v>5</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="13">
+        <v>31284</v>
+      </c>
+      <c r="D7" s="5">
+        <v>50</v>
+      </c>
+      <c r="E7" s="5">
+        <v>68</v>
+      </c>
+      <c r="F7" s="5">
+        <v>50</v>
+      </c>
+      <c r="G7" s="5">
+        <v>78</v>
+      </c>
+      <c r="H7" s="5">
+        <v>34</v>
+      </c>
+      <c r="I7" s="5">
+        <v>71</v>
+      </c>
+      <c r="J7" s="5">
+        <f>SUM(D7:I7)</f>
+        <v>351</v>
+      </c>
+      <c r="K7" s="6">
+        <f t="shared" ref="K7:K12" si="0">AVERAGE(D7:I7)</f>
+        <v>58.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="22.2">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="13">
+        <v>34769</v>
+      </c>
+      <c r="D8" s="5">
+        <v>84</v>
+      </c>
+      <c r="E8" s="5">
+        <v>85</v>
+      </c>
+      <c r="F8" s="5">
+        <v>99</v>
+      </c>
+      <c r="G8" s="5">
+        <v>75</v>
+      </c>
+      <c r="H8" s="5">
+        <v>85</v>
+      </c>
+      <c r="I8" s="5">
+        <v>36</v>
+      </c>
+      <c r="J8" s="5">
+        <f t="shared" ref="J8:J12" si="1">SUM(D8:I8)</f>
+        <v>464</v>
+      </c>
+      <c r="K8" s="6">
+        <f t="shared" si="0"/>
+        <v>77.333333333333329</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="22.2">
+      <c r="A9" s="4">
         <v>7</v>
       </c>
-      <c r="F2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" t="s">
-        <v>4</v>
-      </c>
+      <c r="B9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="13">
+        <v>27587</v>
+      </c>
+      <c r="D9" s="5">
+        <v>31</v>
+      </c>
+      <c r="E9" s="5">
+        <v>95</v>
+      </c>
+      <c r="F9" s="5">
+        <v>90</v>
+      </c>
+      <c r="G9" s="5">
+        <v>71</v>
+      </c>
+      <c r="H9" s="5">
+        <v>31</v>
+      </c>
+      <c r="I9" s="5">
+        <v>82</v>
+      </c>
+      <c r="J9" s="5">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+      <c r="K9" s="6">
+        <f t="shared" si="0"/>
+        <v>66.666666666666671</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="22.2">
+      <c r="A10" s="4">
+        <v>8</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="13">
+        <v>31284</v>
+      </c>
+      <c r="D10" s="5">
+        <v>45</v>
+      </c>
+      <c r="E10" s="5">
+        <v>47</v>
+      </c>
+      <c r="F10" s="5">
+        <v>60</v>
+      </c>
+      <c r="G10" s="5">
+        <v>44</v>
+      </c>
+      <c r="H10" s="5">
+        <v>47</v>
+      </c>
+      <c r="I10" s="5">
+        <v>58</v>
+      </c>
+      <c r="J10" s="5">
+        <f t="shared" si="1"/>
+        <v>301</v>
+      </c>
+      <c r="K10" s="6">
+        <f t="shared" si="0"/>
+        <v>50.166666666666664</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="22.2">
+      <c r="A11" s="4">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="13">
+        <v>34769</v>
+      </c>
+      <c r="D11" s="5">
+        <v>36</v>
+      </c>
+      <c r="E11" s="5">
+        <v>75</v>
+      </c>
+      <c r="F11" s="5">
+        <v>55</v>
+      </c>
+      <c r="G11" s="5">
+        <v>61</v>
+      </c>
+      <c r="H11" s="5">
+        <v>35</v>
+      </c>
+      <c r="I11" s="5">
+        <v>93</v>
+      </c>
+      <c r="J11" s="5">
+        <f t="shared" si="1"/>
+        <v>355</v>
+      </c>
+      <c r="K11" s="6">
+        <f t="shared" si="0"/>
+        <v>59.166666666666664</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="63">
+      <c r="A12" s="10">
+        <v>10</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="13">
+        <v>27587</v>
+      </c>
+      <c r="D12" s="12">
+        <v>45</v>
+      </c>
+      <c r="E12" s="12">
+        <v>49</v>
+      </c>
+      <c r="F12" s="12">
+        <v>38</v>
+      </c>
+      <c r="G12" s="12">
+        <v>84</v>
+      </c>
+      <c r="H12" s="12">
+        <v>37</v>
+      </c>
+      <c r="I12" s="12">
+        <v>56</v>
+      </c>
+      <c r="J12" s="12">
+        <f t="shared" si="1"/>
+        <v>309</v>
+      </c>
+      <c r="K12" s="12">
+        <f t="shared" si="0"/>
+        <v>51.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="22.2">
+      <c r="A13" s="2"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" ht="22.2">
+      <c r="A14" s="2"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>